<commit_message>
Replace bad phones with 'review' in output; remove separate .review files
Invalid/ambiguous phones are replaced with the word 'review' in the number/phone
column. Duplicates are dropped. No separate .review files generated.
</commit_message>
<xml_diff>
--- a/output/campaign_Otros_proyectos.xlsx
+++ b/output/campaign_Otros_proyectos.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2011"/>
+  <dimension ref="A1:C2194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -34603,6 +34603,2385 @@
         </is>
       </c>
     </row>
+    <row r="2012">
+      <c r="A2012" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2012" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2012" t="inlineStr"/>
+    </row>
+    <row r="2013">
+      <c r="A2013" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2013" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2013" t="inlineStr"/>
+    </row>
+    <row r="2014">
+      <c r="A2014" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2014" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2014" t="inlineStr"/>
+    </row>
+    <row r="2015">
+      <c r="A2015" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2015" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2015" t="inlineStr"/>
+    </row>
+    <row r="2016">
+      <c r="A2016" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2016" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2016" t="inlineStr"/>
+    </row>
+    <row r="2017">
+      <c r="A2017" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2017" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2017" t="inlineStr"/>
+    </row>
+    <row r="2018">
+      <c r="A2018" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2018" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2018" t="inlineStr"/>
+    </row>
+    <row r="2019">
+      <c r="A2019" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2019" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2019" t="inlineStr"/>
+    </row>
+    <row r="2020">
+      <c r="A2020" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2020" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2020" t="inlineStr"/>
+    </row>
+    <row r="2021">
+      <c r="A2021" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2021" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2021" t="inlineStr"/>
+    </row>
+    <row r="2022">
+      <c r="A2022" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2022" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2022" t="inlineStr"/>
+    </row>
+    <row r="2023">
+      <c r="A2023" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2023" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2023" t="inlineStr"/>
+    </row>
+    <row r="2024">
+      <c r="A2024" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2024" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2024" t="inlineStr"/>
+    </row>
+    <row r="2025">
+      <c r="A2025" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2025" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2025" t="inlineStr"/>
+    </row>
+    <row r="2026">
+      <c r="A2026" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2026" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2026" t="inlineStr"/>
+    </row>
+    <row r="2027">
+      <c r="A2027" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2027" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2027" t="inlineStr"/>
+    </row>
+    <row r="2028">
+      <c r="A2028" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2028" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2028" t="inlineStr"/>
+    </row>
+    <row r="2029">
+      <c r="A2029" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2029" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2029" t="inlineStr"/>
+    </row>
+    <row r="2030">
+      <c r="A2030" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2030" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2030" t="inlineStr"/>
+    </row>
+    <row r="2031">
+      <c r="A2031" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2031" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2031" t="inlineStr"/>
+    </row>
+    <row r="2032">
+      <c r="A2032" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2032" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2032" t="inlineStr"/>
+    </row>
+    <row r="2033">
+      <c r="A2033" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2033" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2033" t="inlineStr"/>
+    </row>
+    <row r="2034">
+      <c r="A2034" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2034" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2034" t="inlineStr"/>
+    </row>
+    <row r="2035">
+      <c r="A2035" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2035" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2035" t="inlineStr"/>
+    </row>
+    <row r="2036">
+      <c r="A2036" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2036" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2036" t="inlineStr"/>
+    </row>
+    <row r="2037">
+      <c r="A2037" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2037" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2037" t="inlineStr"/>
+    </row>
+    <row r="2038">
+      <c r="A2038" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2038" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2038" t="inlineStr"/>
+    </row>
+    <row r="2039">
+      <c r="A2039" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2039" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2039" t="inlineStr"/>
+    </row>
+    <row r="2040">
+      <c r="A2040" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2040" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2040" t="inlineStr"/>
+    </row>
+    <row r="2041">
+      <c r="A2041" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2041" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2041" t="inlineStr"/>
+    </row>
+    <row r="2042">
+      <c r="A2042" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2042" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2042" t="inlineStr"/>
+    </row>
+    <row r="2043">
+      <c r="A2043" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2043" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2043" t="inlineStr"/>
+    </row>
+    <row r="2044">
+      <c r="A2044" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2044" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2044" t="inlineStr"/>
+    </row>
+    <row r="2045">
+      <c r="A2045" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2045" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2045" t="inlineStr"/>
+    </row>
+    <row r="2046">
+      <c r="A2046" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2046" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2046" t="inlineStr"/>
+    </row>
+    <row r="2047">
+      <c r="A2047" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2047" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2047" t="inlineStr"/>
+    </row>
+    <row r="2048">
+      <c r="A2048" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2048" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2048" t="inlineStr"/>
+    </row>
+    <row r="2049">
+      <c r="A2049" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2049" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2049" t="inlineStr"/>
+    </row>
+    <row r="2050">
+      <c r="A2050" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2050" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2050" t="inlineStr"/>
+    </row>
+    <row r="2051">
+      <c r="A2051" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2051" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2051" t="inlineStr"/>
+    </row>
+    <row r="2052">
+      <c r="A2052" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2052" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2052" t="inlineStr"/>
+    </row>
+    <row r="2053">
+      <c r="A2053" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2053" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2053" t="inlineStr"/>
+    </row>
+    <row r="2054">
+      <c r="A2054" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2054" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2054" t="inlineStr"/>
+    </row>
+    <row r="2055">
+      <c r="A2055" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2055" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2055" t="inlineStr"/>
+    </row>
+    <row r="2056">
+      <c r="A2056" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2056" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2056" t="inlineStr"/>
+    </row>
+    <row r="2057">
+      <c r="A2057" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2057" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2057" t="inlineStr"/>
+    </row>
+    <row r="2058">
+      <c r="A2058" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2058" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2058" t="inlineStr"/>
+    </row>
+    <row r="2059">
+      <c r="A2059" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2059" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2059" t="inlineStr"/>
+    </row>
+    <row r="2060">
+      <c r="A2060" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2060" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2060" t="inlineStr"/>
+    </row>
+    <row r="2061">
+      <c r="A2061" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2061" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2061" t="inlineStr"/>
+    </row>
+    <row r="2062">
+      <c r="A2062" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2062" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2062" t="inlineStr"/>
+    </row>
+    <row r="2063">
+      <c r="A2063" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2063" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2063" t="inlineStr"/>
+    </row>
+    <row r="2064">
+      <c r="A2064" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2064" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2064" t="inlineStr"/>
+    </row>
+    <row r="2065">
+      <c r="A2065" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2065" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2065" t="inlineStr"/>
+    </row>
+    <row r="2066">
+      <c r="A2066" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2066" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2066" t="inlineStr"/>
+    </row>
+    <row r="2067">
+      <c r="A2067" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2067" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2067" t="inlineStr"/>
+    </row>
+    <row r="2068">
+      <c r="A2068" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2068" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2068" t="inlineStr"/>
+    </row>
+    <row r="2069">
+      <c r="A2069" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2069" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2069" t="inlineStr"/>
+    </row>
+    <row r="2070">
+      <c r="A2070" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2070" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2070" t="inlineStr"/>
+    </row>
+    <row r="2071">
+      <c r="A2071" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2071" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2071" t="inlineStr"/>
+    </row>
+    <row r="2072">
+      <c r="A2072" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2072" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2072" t="inlineStr"/>
+    </row>
+    <row r="2073">
+      <c r="A2073" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2073" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2073" t="inlineStr"/>
+    </row>
+    <row r="2074">
+      <c r="A2074" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2074" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2074" t="inlineStr"/>
+    </row>
+    <row r="2075">
+      <c r="A2075" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2075" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2075" t="inlineStr"/>
+    </row>
+    <row r="2076">
+      <c r="A2076" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2076" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2076" t="inlineStr"/>
+    </row>
+    <row r="2077">
+      <c r="A2077" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2077" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2077" t="inlineStr"/>
+    </row>
+    <row r="2078">
+      <c r="A2078" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2078" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2078" t="inlineStr"/>
+    </row>
+    <row r="2079">
+      <c r="A2079" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2079" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2079" t="inlineStr"/>
+    </row>
+    <row r="2080">
+      <c r="A2080" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2080" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2080" t="inlineStr"/>
+    </row>
+    <row r="2081">
+      <c r="A2081" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2081" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2081" t="inlineStr"/>
+    </row>
+    <row r="2082">
+      <c r="A2082" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2082" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2082" t="inlineStr"/>
+    </row>
+    <row r="2083">
+      <c r="A2083" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2083" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2083" t="inlineStr"/>
+    </row>
+    <row r="2084">
+      <c r="A2084" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2084" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2084" t="inlineStr"/>
+    </row>
+    <row r="2085">
+      <c r="A2085" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2085" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2085" t="inlineStr"/>
+    </row>
+    <row r="2086">
+      <c r="A2086" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2086" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2086" t="inlineStr"/>
+    </row>
+    <row r="2087">
+      <c r="A2087" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2087" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2087" t="inlineStr"/>
+    </row>
+    <row r="2088">
+      <c r="A2088" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2088" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2088" t="inlineStr"/>
+    </row>
+    <row r="2089">
+      <c r="A2089" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2089" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2089" t="inlineStr"/>
+    </row>
+    <row r="2090">
+      <c r="A2090" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2090" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2090" t="inlineStr"/>
+    </row>
+    <row r="2091">
+      <c r="A2091" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2091" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2091" t="inlineStr"/>
+    </row>
+    <row r="2092">
+      <c r="A2092" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2092" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2092" t="inlineStr"/>
+    </row>
+    <row r="2093">
+      <c r="A2093" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2093" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2093" t="inlineStr"/>
+    </row>
+    <row r="2094">
+      <c r="A2094" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2094" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2094" t="inlineStr"/>
+    </row>
+    <row r="2095">
+      <c r="A2095" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2095" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2095" t="inlineStr"/>
+    </row>
+    <row r="2096">
+      <c r="A2096" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2096" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2096" t="inlineStr"/>
+    </row>
+    <row r="2097">
+      <c r="A2097" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2097" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2097" t="inlineStr"/>
+    </row>
+    <row r="2098">
+      <c r="A2098" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2098" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2098" t="inlineStr"/>
+    </row>
+    <row r="2099">
+      <c r="A2099" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2099" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2099" t="inlineStr"/>
+    </row>
+    <row r="2100">
+      <c r="A2100" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2100" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2100" t="inlineStr"/>
+    </row>
+    <row r="2101">
+      <c r="A2101" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2101" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2101" t="inlineStr"/>
+    </row>
+    <row r="2102">
+      <c r="A2102" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2102" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2102" t="inlineStr"/>
+    </row>
+    <row r="2103">
+      <c r="A2103" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2103" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2103" t="inlineStr"/>
+    </row>
+    <row r="2104">
+      <c r="A2104" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2104" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2104" t="inlineStr"/>
+    </row>
+    <row r="2105">
+      <c r="A2105" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2105" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2105" t="inlineStr"/>
+    </row>
+    <row r="2106">
+      <c r="A2106" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2106" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2106" t="inlineStr"/>
+    </row>
+    <row r="2107">
+      <c r="A2107" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2107" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2107" t="inlineStr"/>
+    </row>
+    <row r="2108">
+      <c r="A2108" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2108" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2108" t="inlineStr"/>
+    </row>
+    <row r="2109">
+      <c r="A2109" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2109" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2109" t="inlineStr"/>
+    </row>
+    <row r="2110">
+      <c r="A2110" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2110" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2110" t="inlineStr"/>
+    </row>
+    <row r="2111">
+      <c r="A2111" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2111" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2111" t="inlineStr"/>
+    </row>
+    <row r="2112">
+      <c r="A2112" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2112" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2112" t="inlineStr"/>
+    </row>
+    <row r="2113">
+      <c r="A2113" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2113" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2113" t="inlineStr"/>
+    </row>
+    <row r="2114">
+      <c r="A2114" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2114" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2114" t="inlineStr"/>
+    </row>
+    <row r="2115">
+      <c r="A2115" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2115" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2115" t="inlineStr"/>
+    </row>
+    <row r="2116">
+      <c r="A2116" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2116" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2116" t="inlineStr"/>
+    </row>
+    <row r="2117">
+      <c r="A2117" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2117" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2117" t="inlineStr"/>
+    </row>
+    <row r="2118">
+      <c r="A2118" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2118" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2118" t="inlineStr"/>
+    </row>
+    <row r="2119">
+      <c r="A2119" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2119" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2119" t="inlineStr"/>
+    </row>
+    <row r="2120">
+      <c r="A2120" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2120" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2120" t="inlineStr"/>
+    </row>
+    <row r="2121">
+      <c r="A2121" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2121" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2121" t="inlineStr"/>
+    </row>
+    <row r="2122">
+      <c r="A2122" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2122" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2122" t="inlineStr"/>
+    </row>
+    <row r="2123">
+      <c r="A2123" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2123" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2123" t="inlineStr"/>
+    </row>
+    <row r="2124">
+      <c r="A2124" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2124" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2124" t="inlineStr"/>
+    </row>
+    <row r="2125">
+      <c r="A2125" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2125" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2125" t="inlineStr"/>
+    </row>
+    <row r="2126">
+      <c r="A2126" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2126" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2126" t="inlineStr"/>
+    </row>
+    <row r="2127">
+      <c r="A2127" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2127" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2127" t="inlineStr"/>
+    </row>
+    <row r="2128">
+      <c r="A2128" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2128" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2128" t="inlineStr"/>
+    </row>
+    <row r="2129">
+      <c r="A2129" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2129" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2129" t="inlineStr"/>
+    </row>
+    <row r="2130">
+      <c r="A2130" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2130" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2130" t="inlineStr"/>
+    </row>
+    <row r="2131">
+      <c r="A2131" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2131" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2131" t="inlineStr"/>
+    </row>
+    <row r="2132">
+      <c r="A2132" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2132" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2132" t="inlineStr"/>
+    </row>
+    <row r="2133">
+      <c r="A2133" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2133" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2133" t="inlineStr"/>
+    </row>
+    <row r="2134">
+      <c r="A2134" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2134" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2134" t="inlineStr"/>
+    </row>
+    <row r="2135">
+      <c r="A2135" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2135" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2135" t="inlineStr"/>
+    </row>
+    <row r="2136">
+      <c r="A2136" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2136" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2136" t="inlineStr"/>
+    </row>
+    <row r="2137">
+      <c r="A2137" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2137" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2137" t="inlineStr"/>
+    </row>
+    <row r="2138">
+      <c r="A2138" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2138" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2138" t="inlineStr"/>
+    </row>
+    <row r="2139">
+      <c r="A2139" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2139" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2139" t="inlineStr"/>
+    </row>
+    <row r="2140">
+      <c r="A2140" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2140" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2140" t="inlineStr"/>
+    </row>
+    <row r="2141">
+      <c r="A2141" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2141" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2141" t="inlineStr"/>
+    </row>
+    <row r="2142">
+      <c r="A2142" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2142" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2142" t="inlineStr"/>
+    </row>
+    <row r="2143">
+      <c r="A2143" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2143" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2143" t="inlineStr"/>
+    </row>
+    <row r="2144">
+      <c r="A2144" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2144" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2144" t="inlineStr"/>
+    </row>
+    <row r="2145">
+      <c r="A2145" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2145" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2145" t="inlineStr"/>
+    </row>
+    <row r="2146">
+      <c r="A2146" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2146" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2146" t="inlineStr"/>
+    </row>
+    <row r="2147">
+      <c r="A2147" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2147" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2147" t="inlineStr"/>
+    </row>
+    <row r="2148">
+      <c r="A2148" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2148" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2148" t="inlineStr"/>
+    </row>
+    <row r="2149">
+      <c r="A2149" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2149" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2149" t="inlineStr"/>
+    </row>
+    <row r="2150">
+      <c r="A2150" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2150" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2150" t="inlineStr"/>
+    </row>
+    <row r="2151">
+      <c r="A2151" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2151" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2151" t="inlineStr"/>
+    </row>
+    <row r="2152">
+      <c r="A2152" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2152" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2152" t="inlineStr"/>
+    </row>
+    <row r="2153">
+      <c r="A2153" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2153" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2153" t="inlineStr"/>
+    </row>
+    <row r="2154">
+      <c r="A2154" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2154" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2154" t="inlineStr"/>
+    </row>
+    <row r="2155">
+      <c r="A2155" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2155" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2155" t="inlineStr"/>
+    </row>
+    <row r="2156">
+      <c r="A2156" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2156" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2156" t="inlineStr"/>
+    </row>
+    <row r="2157">
+      <c r="A2157" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2157" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2157" t="inlineStr"/>
+    </row>
+    <row r="2158">
+      <c r="A2158" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2158" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2158" t="inlineStr"/>
+    </row>
+    <row r="2159">
+      <c r="A2159" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2159" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2159" t="inlineStr"/>
+    </row>
+    <row r="2160">
+      <c r="A2160" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2160" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2160" t="inlineStr"/>
+    </row>
+    <row r="2161">
+      <c r="A2161" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2161" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2161" t="inlineStr"/>
+    </row>
+    <row r="2162">
+      <c r="A2162" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2162" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2162" t="inlineStr"/>
+    </row>
+    <row r="2163">
+      <c r="A2163" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2163" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2163" t="inlineStr"/>
+    </row>
+    <row r="2164">
+      <c r="A2164" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2164" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2164" t="inlineStr"/>
+    </row>
+    <row r="2165">
+      <c r="A2165" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2165" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2165" t="inlineStr"/>
+    </row>
+    <row r="2166">
+      <c r="A2166" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2166" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2166" t="inlineStr"/>
+    </row>
+    <row r="2167">
+      <c r="A2167" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2167" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2167" t="inlineStr"/>
+    </row>
+    <row r="2168">
+      <c r="A2168" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2168" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2168" t="inlineStr"/>
+    </row>
+    <row r="2169">
+      <c r="A2169" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2169" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2169" t="inlineStr"/>
+    </row>
+    <row r="2170">
+      <c r="A2170" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2170" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2170" t="inlineStr"/>
+    </row>
+    <row r="2171">
+      <c r="A2171" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2171" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2171" t="inlineStr"/>
+    </row>
+    <row r="2172">
+      <c r="A2172" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2172" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2172" t="inlineStr"/>
+    </row>
+    <row r="2173">
+      <c r="A2173" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2173" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2173" t="inlineStr"/>
+    </row>
+    <row r="2174">
+      <c r="A2174" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2174" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2174" t="inlineStr"/>
+    </row>
+    <row r="2175">
+      <c r="A2175" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2175" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2175" t="inlineStr"/>
+    </row>
+    <row r="2176">
+      <c r="A2176" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2176" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2176" t="inlineStr"/>
+    </row>
+    <row r="2177">
+      <c r="A2177" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2177" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2177" t="inlineStr"/>
+    </row>
+    <row r="2178">
+      <c r="A2178" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2178" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2178" t="inlineStr"/>
+    </row>
+    <row r="2179">
+      <c r="A2179" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2179" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2179" t="inlineStr"/>
+    </row>
+    <row r="2180">
+      <c r="A2180" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2180" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2180" t="inlineStr"/>
+    </row>
+    <row r="2181">
+      <c r="A2181" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2181" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2181" t="inlineStr"/>
+    </row>
+    <row r="2182">
+      <c r="A2182" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2182" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2182" t="inlineStr"/>
+    </row>
+    <row r="2183">
+      <c r="A2183" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2183" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2183" t="inlineStr"/>
+    </row>
+    <row r="2184">
+      <c r="A2184" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2184" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2184" t="inlineStr"/>
+    </row>
+    <row r="2185">
+      <c r="A2185" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2185" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2185" t="inlineStr"/>
+    </row>
+    <row r="2186">
+      <c r="A2186" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2186" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2186" t="inlineStr"/>
+    </row>
+    <row r="2187">
+      <c r="A2187" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2187" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2187" t="inlineStr"/>
+    </row>
+    <row r="2188">
+      <c r="A2188" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2188" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2188" t="inlineStr"/>
+    </row>
+    <row r="2189">
+      <c r="A2189" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2189" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2189" t="inlineStr"/>
+    </row>
+    <row r="2190">
+      <c r="A2190" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2190" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2190" t="inlineStr"/>
+    </row>
+    <row r="2191">
+      <c r="A2191" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2191" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2191" t="inlineStr"/>
+    </row>
+    <row r="2192">
+      <c r="A2192" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2192" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2192" t="inlineStr"/>
+    </row>
+    <row r="2193">
+      <c r="A2193" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2193" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2193" t="inlineStr"/>
+    </row>
+    <row r="2194">
+      <c r="A2194" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2194" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2194" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Route bad phones to 'review' inline; always 4 output files, no .review files
</commit_message>
<xml_diff>
--- a/output/campaign_Otros_proyectos.xlsx
+++ b/output/campaign_Otros_proyectos.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2011"/>
+  <dimension ref="A1:C2194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -34603,6 +34603,2385 @@
         </is>
       </c>
     </row>
+    <row r="2012">
+      <c r="A2012" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2012" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2012" t="inlineStr"/>
+    </row>
+    <row r="2013">
+      <c r="A2013" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2013" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2013" t="inlineStr"/>
+    </row>
+    <row r="2014">
+      <c r="A2014" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2014" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2014" t="inlineStr"/>
+    </row>
+    <row r="2015">
+      <c r="A2015" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2015" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2015" t="inlineStr"/>
+    </row>
+    <row r="2016">
+      <c r="A2016" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2016" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2016" t="inlineStr"/>
+    </row>
+    <row r="2017">
+      <c r="A2017" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2017" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2017" t="inlineStr"/>
+    </row>
+    <row r="2018">
+      <c r="A2018" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2018" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2018" t="inlineStr"/>
+    </row>
+    <row r="2019">
+      <c r="A2019" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2019" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2019" t="inlineStr"/>
+    </row>
+    <row r="2020">
+      <c r="A2020" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2020" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2020" t="inlineStr"/>
+    </row>
+    <row r="2021">
+      <c r="A2021" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2021" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2021" t="inlineStr"/>
+    </row>
+    <row r="2022">
+      <c r="A2022" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2022" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2022" t="inlineStr"/>
+    </row>
+    <row r="2023">
+      <c r="A2023" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2023" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2023" t="inlineStr"/>
+    </row>
+    <row r="2024">
+      <c r="A2024" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2024" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2024" t="inlineStr"/>
+    </row>
+    <row r="2025">
+      <c r="A2025" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2025" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2025" t="inlineStr"/>
+    </row>
+    <row r="2026">
+      <c r="A2026" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2026" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2026" t="inlineStr"/>
+    </row>
+    <row r="2027">
+      <c r="A2027" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2027" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2027" t="inlineStr"/>
+    </row>
+    <row r="2028">
+      <c r="A2028" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2028" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2028" t="inlineStr"/>
+    </row>
+    <row r="2029">
+      <c r="A2029" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2029" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2029" t="inlineStr"/>
+    </row>
+    <row r="2030">
+      <c r="A2030" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2030" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2030" t="inlineStr"/>
+    </row>
+    <row r="2031">
+      <c r="A2031" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2031" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2031" t="inlineStr"/>
+    </row>
+    <row r="2032">
+      <c r="A2032" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2032" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2032" t="inlineStr"/>
+    </row>
+    <row r="2033">
+      <c r="A2033" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2033" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2033" t="inlineStr"/>
+    </row>
+    <row r="2034">
+      <c r="A2034" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2034" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2034" t="inlineStr"/>
+    </row>
+    <row r="2035">
+      <c r="A2035" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2035" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2035" t="inlineStr"/>
+    </row>
+    <row r="2036">
+      <c r="A2036" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2036" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2036" t="inlineStr"/>
+    </row>
+    <row r="2037">
+      <c r="A2037" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2037" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2037" t="inlineStr"/>
+    </row>
+    <row r="2038">
+      <c r="A2038" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2038" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2038" t="inlineStr"/>
+    </row>
+    <row r="2039">
+      <c r="A2039" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2039" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2039" t="inlineStr"/>
+    </row>
+    <row r="2040">
+      <c r="A2040" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2040" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2040" t="inlineStr"/>
+    </row>
+    <row r="2041">
+      <c r="A2041" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2041" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2041" t="inlineStr"/>
+    </row>
+    <row r="2042">
+      <c r="A2042" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2042" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2042" t="inlineStr"/>
+    </row>
+    <row r="2043">
+      <c r="A2043" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2043" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2043" t="inlineStr"/>
+    </row>
+    <row r="2044">
+      <c r="A2044" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2044" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2044" t="inlineStr"/>
+    </row>
+    <row r="2045">
+      <c r="A2045" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2045" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2045" t="inlineStr"/>
+    </row>
+    <row r="2046">
+      <c r="A2046" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2046" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2046" t="inlineStr"/>
+    </row>
+    <row r="2047">
+      <c r="A2047" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2047" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2047" t="inlineStr"/>
+    </row>
+    <row r="2048">
+      <c r="A2048" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2048" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2048" t="inlineStr"/>
+    </row>
+    <row r="2049">
+      <c r="A2049" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2049" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2049" t="inlineStr"/>
+    </row>
+    <row r="2050">
+      <c r="A2050" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2050" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2050" t="inlineStr"/>
+    </row>
+    <row r="2051">
+      <c r="A2051" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2051" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2051" t="inlineStr"/>
+    </row>
+    <row r="2052">
+      <c r="A2052" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2052" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2052" t="inlineStr"/>
+    </row>
+    <row r="2053">
+      <c r="A2053" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2053" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2053" t="inlineStr"/>
+    </row>
+    <row r="2054">
+      <c r="A2054" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2054" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2054" t="inlineStr"/>
+    </row>
+    <row r="2055">
+      <c r="A2055" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2055" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2055" t="inlineStr"/>
+    </row>
+    <row r="2056">
+      <c r="A2056" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2056" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2056" t="inlineStr"/>
+    </row>
+    <row r="2057">
+      <c r="A2057" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2057" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2057" t="inlineStr"/>
+    </row>
+    <row r="2058">
+      <c r="A2058" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2058" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2058" t="inlineStr"/>
+    </row>
+    <row r="2059">
+      <c r="A2059" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2059" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2059" t="inlineStr"/>
+    </row>
+    <row r="2060">
+      <c r="A2060" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2060" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2060" t="inlineStr"/>
+    </row>
+    <row r="2061">
+      <c r="A2061" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2061" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2061" t="inlineStr"/>
+    </row>
+    <row r="2062">
+      <c r="A2062" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2062" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2062" t="inlineStr"/>
+    </row>
+    <row r="2063">
+      <c r="A2063" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2063" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2063" t="inlineStr"/>
+    </row>
+    <row r="2064">
+      <c r="A2064" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2064" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2064" t="inlineStr"/>
+    </row>
+    <row r="2065">
+      <c r="A2065" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2065" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2065" t="inlineStr"/>
+    </row>
+    <row r="2066">
+      <c r="A2066" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2066" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2066" t="inlineStr"/>
+    </row>
+    <row r="2067">
+      <c r="A2067" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2067" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2067" t="inlineStr"/>
+    </row>
+    <row r="2068">
+      <c r="A2068" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2068" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2068" t="inlineStr"/>
+    </row>
+    <row r="2069">
+      <c r="A2069" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2069" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2069" t="inlineStr"/>
+    </row>
+    <row r="2070">
+      <c r="A2070" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2070" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2070" t="inlineStr"/>
+    </row>
+    <row r="2071">
+      <c r="A2071" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2071" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2071" t="inlineStr"/>
+    </row>
+    <row r="2072">
+      <c r="A2072" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2072" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2072" t="inlineStr"/>
+    </row>
+    <row r="2073">
+      <c r="A2073" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2073" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2073" t="inlineStr"/>
+    </row>
+    <row r="2074">
+      <c r="A2074" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2074" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2074" t="inlineStr"/>
+    </row>
+    <row r="2075">
+      <c r="A2075" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2075" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2075" t="inlineStr"/>
+    </row>
+    <row r="2076">
+      <c r="A2076" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2076" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2076" t="inlineStr"/>
+    </row>
+    <row r="2077">
+      <c r="A2077" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2077" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2077" t="inlineStr"/>
+    </row>
+    <row r="2078">
+      <c r="A2078" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2078" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2078" t="inlineStr"/>
+    </row>
+    <row r="2079">
+      <c r="A2079" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2079" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2079" t="inlineStr"/>
+    </row>
+    <row r="2080">
+      <c r="A2080" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2080" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2080" t="inlineStr"/>
+    </row>
+    <row r="2081">
+      <c r="A2081" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2081" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2081" t="inlineStr"/>
+    </row>
+    <row r="2082">
+      <c r="A2082" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2082" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2082" t="inlineStr"/>
+    </row>
+    <row r="2083">
+      <c r="A2083" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2083" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2083" t="inlineStr"/>
+    </row>
+    <row r="2084">
+      <c r="A2084" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2084" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2084" t="inlineStr"/>
+    </row>
+    <row r="2085">
+      <c r="A2085" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2085" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2085" t="inlineStr"/>
+    </row>
+    <row r="2086">
+      <c r="A2086" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2086" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2086" t="inlineStr"/>
+    </row>
+    <row r="2087">
+      <c r="A2087" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2087" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2087" t="inlineStr"/>
+    </row>
+    <row r="2088">
+      <c r="A2088" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2088" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2088" t="inlineStr"/>
+    </row>
+    <row r="2089">
+      <c r="A2089" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2089" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2089" t="inlineStr"/>
+    </row>
+    <row r="2090">
+      <c r="A2090" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2090" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2090" t="inlineStr"/>
+    </row>
+    <row r="2091">
+      <c r="A2091" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2091" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2091" t="inlineStr"/>
+    </row>
+    <row r="2092">
+      <c r="A2092" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2092" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2092" t="inlineStr"/>
+    </row>
+    <row r="2093">
+      <c r="A2093" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2093" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2093" t="inlineStr"/>
+    </row>
+    <row r="2094">
+      <c r="A2094" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2094" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2094" t="inlineStr"/>
+    </row>
+    <row r="2095">
+      <c r="A2095" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2095" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2095" t="inlineStr"/>
+    </row>
+    <row r="2096">
+      <c r="A2096" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2096" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2096" t="inlineStr"/>
+    </row>
+    <row r="2097">
+      <c r="A2097" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2097" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2097" t="inlineStr"/>
+    </row>
+    <row r="2098">
+      <c r="A2098" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2098" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2098" t="inlineStr"/>
+    </row>
+    <row r="2099">
+      <c r="A2099" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2099" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2099" t="inlineStr"/>
+    </row>
+    <row r="2100">
+      <c r="A2100" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2100" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2100" t="inlineStr"/>
+    </row>
+    <row r="2101">
+      <c r="A2101" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2101" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2101" t="inlineStr"/>
+    </row>
+    <row r="2102">
+      <c r="A2102" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2102" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2102" t="inlineStr"/>
+    </row>
+    <row r="2103">
+      <c r="A2103" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2103" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2103" t="inlineStr"/>
+    </row>
+    <row r="2104">
+      <c r="A2104" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2104" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2104" t="inlineStr"/>
+    </row>
+    <row r="2105">
+      <c r="A2105" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2105" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2105" t="inlineStr"/>
+    </row>
+    <row r="2106">
+      <c r="A2106" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2106" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2106" t="inlineStr"/>
+    </row>
+    <row r="2107">
+      <c r="A2107" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2107" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2107" t="inlineStr"/>
+    </row>
+    <row r="2108">
+      <c r="A2108" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2108" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2108" t="inlineStr"/>
+    </row>
+    <row r="2109">
+      <c r="A2109" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2109" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2109" t="inlineStr"/>
+    </row>
+    <row r="2110">
+      <c r="A2110" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2110" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2110" t="inlineStr"/>
+    </row>
+    <row r="2111">
+      <c r="A2111" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2111" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2111" t="inlineStr"/>
+    </row>
+    <row r="2112">
+      <c r="A2112" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2112" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2112" t="inlineStr"/>
+    </row>
+    <row r="2113">
+      <c r="A2113" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2113" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2113" t="inlineStr"/>
+    </row>
+    <row r="2114">
+      <c r="A2114" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2114" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2114" t="inlineStr"/>
+    </row>
+    <row r="2115">
+      <c r="A2115" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2115" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2115" t="inlineStr"/>
+    </row>
+    <row r="2116">
+      <c r="A2116" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2116" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2116" t="inlineStr"/>
+    </row>
+    <row r="2117">
+      <c r="A2117" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2117" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2117" t="inlineStr"/>
+    </row>
+    <row r="2118">
+      <c r="A2118" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2118" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2118" t="inlineStr"/>
+    </row>
+    <row r="2119">
+      <c r="A2119" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2119" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2119" t="inlineStr"/>
+    </row>
+    <row r="2120">
+      <c r="A2120" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2120" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2120" t="inlineStr"/>
+    </row>
+    <row r="2121">
+      <c r="A2121" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2121" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2121" t="inlineStr"/>
+    </row>
+    <row r="2122">
+      <c r="A2122" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2122" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2122" t="inlineStr"/>
+    </row>
+    <row r="2123">
+      <c r="A2123" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2123" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2123" t="inlineStr"/>
+    </row>
+    <row r="2124">
+      <c r="A2124" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2124" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2124" t="inlineStr"/>
+    </row>
+    <row r="2125">
+      <c r="A2125" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2125" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2125" t="inlineStr"/>
+    </row>
+    <row r="2126">
+      <c r="A2126" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2126" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2126" t="inlineStr"/>
+    </row>
+    <row r="2127">
+      <c r="A2127" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2127" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2127" t="inlineStr"/>
+    </row>
+    <row r="2128">
+      <c r="A2128" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2128" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2128" t="inlineStr"/>
+    </row>
+    <row r="2129">
+      <c r="A2129" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2129" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2129" t="inlineStr"/>
+    </row>
+    <row r="2130">
+      <c r="A2130" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2130" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2130" t="inlineStr"/>
+    </row>
+    <row r="2131">
+      <c r="A2131" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2131" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2131" t="inlineStr"/>
+    </row>
+    <row r="2132">
+      <c r="A2132" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2132" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2132" t="inlineStr"/>
+    </row>
+    <row r="2133">
+      <c r="A2133" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2133" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2133" t="inlineStr"/>
+    </row>
+    <row r="2134">
+      <c r="A2134" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2134" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2134" t="inlineStr"/>
+    </row>
+    <row r="2135">
+      <c r="A2135" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2135" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2135" t="inlineStr"/>
+    </row>
+    <row r="2136">
+      <c r="A2136" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2136" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2136" t="inlineStr"/>
+    </row>
+    <row r="2137">
+      <c r="A2137" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2137" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2137" t="inlineStr"/>
+    </row>
+    <row r="2138">
+      <c r="A2138" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2138" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2138" t="inlineStr"/>
+    </row>
+    <row r="2139">
+      <c r="A2139" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2139" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2139" t="inlineStr"/>
+    </row>
+    <row r="2140">
+      <c r="A2140" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2140" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2140" t="inlineStr"/>
+    </row>
+    <row r="2141">
+      <c r="A2141" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2141" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2141" t="inlineStr"/>
+    </row>
+    <row r="2142">
+      <c r="A2142" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2142" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2142" t="inlineStr"/>
+    </row>
+    <row r="2143">
+      <c r="A2143" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2143" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2143" t="inlineStr"/>
+    </row>
+    <row r="2144">
+      <c r="A2144" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2144" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2144" t="inlineStr"/>
+    </row>
+    <row r="2145">
+      <c r="A2145" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2145" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2145" t="inlineStr"/>
+    </row>
+    <row r="2146">
+      <c r="A2146" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2146" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2146" t="inlineStr"/>
+    </row>
+    <row r="2147">
+      <c r="A2147" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2147" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2147" t="inlineStr"/>
+    </row>
+    <row r="2148">
+      <c r="A2148" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2148" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2148" t="inlineStr"/>
+    </row>
+    <row r="2149">
+      <c r="A2149" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2149" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2149" t="inlineStr"/>
+    </row>
+    <row r="2150">
+      <c r="A2150" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2150" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2150" t="inlineStr"/>
+    </row>
+    <row r="2151">
+      <c r="A2151" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2151" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2151" t="inlineStr"/>
+    </row>
+    <row r="2152">
+      <c r="A2152" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2152" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2152" t="inlineStr"/>
+    </row>
+    <row r="2153">
+      <c r="A2153" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2153" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2153" t="inlineStr"/>
+    </row>
+    <row r="2154">
+      <c r="A2154" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2154" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2154" t="inlineStr"/>
+    </row>
+    <row r="2155">
+      <c r="A2155" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2155" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2155" t="inlineStr"/>
+    </row>
+    <row r="2156">
+      <c r="A2156" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2156" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2156" t="inlineStr"/>
+    </row>
+    <row r="2157">
+      <c r="A2157" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2157" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2157" t="inlineStr"/>
+    </row>
+    <row r="2158">
+      <c r="A2158" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2158" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2158" t="inlineStr"/>
+    </row>
+    <row r="2159">
+      <c r="A2159" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2159" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2159" t="inlineStr"/>
+    </row>
+    <row r="2160">
+      <c r="A2160" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2160" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2160" t="inlineStr"/>
+    </row>
+    <row r="2161">
+      <c r="A2161" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2161" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2161" t="inlineStr"/>
+    </row>
+    <row r="2162">
+      <c r="A2162" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2162" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2162" t="inlineStr"/>
+    </row>
+    <row r="2163">
+      <c r="A2163" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2163" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2163" t="inlineStr"/>
+    </row>
+    <row r="2164">
+      <c r="A2164" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2164" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2164" t="inlineStr"/>
+    </row>
+    <row r="2165">
+      <c r="A2165" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2165" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2165" t="inlineStr"/>
+    </row>
+    <row r="2166">
+      <c r="A2166" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2166" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2166" t="inlineStr"/>
+    </row>
+    <row r="2167">
+      <c r="A2167" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2167" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2167" t="inlineStr"/>
+    </row>
+    <row r="2168">
+      <c r="A2168" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2168" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2168" t="inlineStr"/>
+    </row>
+    <row r="2169">
+      <c r="A2169" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2169" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2169" t="inlineStr"/>
+    </row>
+    <row r="2170">
+      <c r="A2170" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2170" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2170" t="inlineStr"/>
+    </row>
+    <row r="2171">
+      <c r="A2171" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2171" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2171" t="inlineStr"/>
+    </row>
+    <row r="2172">
+      <c r="A2172" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2172" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2172" t="inlineStr"/>
+    </row>
+    <row r="2173">
+      <c r="A2173" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2173" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2173" t="inlineStr"/>
+    </row>
+    <row r="2174">
+      <c r="A2174" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2174" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2174" t="inlineStr"/>
+    </row>
+    <row r="2175">
+      <c r="A2175" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2175" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2175" t="inlineStr"/>
+    </row>
+    <row r="2176">
+      <c r="A2176" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2176" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2176" t="inlineStr"/>
+    </row>
+    <row r="2177">
+      <c r="A2177" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2177" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2177" t="inlineStr"/>
+    </row>
+    <row r="2178">
+      <c r="A2178" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2178" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2178" t="inlineStr"/>
+    </row>
+    <row r="2179">
+      <c r="A2179" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2179" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2179" t="inlineStr"/>
+    </row>
+    <row r="2180">
+      <c r="A2180" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2180" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2180" t="inlineStr"/>
+    </row>
+    <row r="2181">
+      <c r="A2181" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2181" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2181" t="inlineStr"/>
+    </row>
+    <row r="2182">
+      <c r="A2182" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2182" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2182" t="inlineStr"/>
+    </row>
+    <row r="2183">
+      <c r="A2183" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2183" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2183" t="inlineStr"/>
+    </row>
+    <row r="2184">
+      <c r="A2184" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2184" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2184" t="inlineStr"/>
+    </row>
+    <row r="2185">
+      <c r="A2185" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2185" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2185" t="inlineStr"/>
+    </row>
+    <row r="2186">
+      <c r="A2186" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2186" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2186" t="inlineStr"/>
+    </row>
+    <row r="2187">
+      <c r="A2187" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2187" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2187" t="inlineStr"/>
+    </row>
+    <row r="2188">
+      <c r="A2188" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2188" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2188" t="inlineStr"/>
+    </row>
+    <row r="2189">
+      <c r="A2189" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2189" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2189" t="inlineStr"/>
+    </row>
+    <row r="2190">
+      <c r="A2190" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2190" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2190" t="inlineStr"/>
+    </row>
+    <row r="2191">
+      <c r="A2191" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2191" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2191" t="inlineStr"/>
+    </row>
+    <row r="2192">
+      <c r="A2192" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2192" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2192" t="inlineStr"/>
+    </row>
+    <row r="2193">
+      <c r="A2193" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2193" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2193" t="inlineStr"/>
+    </row>
+    <row r="2194">
+      <c r="A2194" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B2194" t="inlineStr">
+        <is>
+          <t>nan nan</t>
+        </is>
+      </c>
+      <c r="C2194" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix voice_model_selection lookup, drop bad-phone rows entirely
- voice_model_selection now looked up from customers template by phone
- Invalid/ambiguous phones dropped from output entirely (no 'review' rows)
- Removes nan nan rows from campaign output
- Always exactly 4 output files
</commit_message>
<xml_diff>
--- a/output/campaign_Otros_proyectos.xlsx
+++ b/output/campaign_Otros_proyectos.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2194"/>
+  <dimension ref="A1:C2011"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -34603,2385 +34603,6 @@
         </is>
       </c>
     </row>
-    <row r="2012">
-      <c r="A2012" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2012" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2012" t="inlineStr"/>
-    </row>
-    <row r="2013">
-      <c r="A2013" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2013" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2013" t="inlineStr"/>
-    </row>
-    <row r="2014">
-      <c r="A2014" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2014" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2014" t="inlineStr"/>
-    </row>
-    <row r="2015">
-      <c r="A2015" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2015" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2015" t="inlineStr"/>
-    </row>
-    <row r="2016">
-      <c r="A2016" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2016" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2016" t="inlineStr"/>
-    </row>
-    <row r="2017">
-      <c r="A2017" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2017" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2017" t="inlineStr"/>
-    </row>
-    <row r="2018">
-      <c r="A2018" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2018" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2018" t="inlineStr"/>
-    </row>
-    <row r="2019">
-      <c r="A2019" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2019" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2019" t="inlineStr"/>
-    </row>
-    <row r="2020">
-      <c r="A2020" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2020" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2020" t="inlineStr"/>
-    </row>
-    <row r="2021">
-      <c r="A2021" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2021" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2021" t="inlineStr"/>
-    </row>
-    <row r="2022">
-      <c r="A2022" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2022" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2022" t="inlineStr"/>
-    </row>
-    <row r="2023">
-      <c r="A2023" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2023" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2023" t="inlineStr"/>
-    </row>
-    <row r="2024">
-      <c r="A2024" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2024" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2024" t="inlineStr"/>
-    </row>
-    <row r="2025">
-      <c r="A2025" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2025" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2025" t="inlineStr"/>
-    </row>
-    <row r="2026">
-      <c r="A2026" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2026" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2026" t="inlineStr"/>
-    </row>
-    <row r="2027">
-      <c r="A2027" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2027" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2027" t="inlineStr"/>
-    </row>
-    <row r="2028">
-      <c r="A2028" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2028" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2028" t="inlineStr"/>
-    </row>
-    <row r="2029">
-      <c r="A2029" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2029" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2029" t="inlineStr"/>
-    </row>
-    <row r="2030">
-      <c r="A2030" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2030" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2030" t="inlineStr"/>
-    </row>
-    <row r="2031">
-      <c r="A2031" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2031" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2031" t="inlineStr"/>
-    </row>
-    <row r="2032">
-      <c r="A2032" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2032" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2032" t="inlineStr"/>
-    </row>
-    <row r="2033">
-      <c r="A2033" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2033" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2033" t="inlineStr"/>
-    </row>
-    <row r="2034">
-      <c r="A2034" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2034" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2034" t="inlineStr"/>
-    </row>
-    <row r="2035">
-      <c r="A2035" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2035" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2035" t="inlineStr"/>
-    </row>
-    <row r="2036">
-      <c r="A2036" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2036" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2036" t="inlineStr"/>
-    </row>
-    <row r="2037">
-      <c r="A2037" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2037" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2037" t="inlineStr"/>
-    </row>
-    <row r="2038">
-      <c r="A2038" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2038" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2038" t="inlineStr"/>
-    </row>
-    <row r="2039">
-      <c r="A2039" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2039" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2039" t="inlineStr"/>
-    </row>
-    <row r="2040">
-      <c r="A2040" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2040" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2040" t="inlineStr"/>
-    </row>
-    <row r="2041">
-      <c r="A2041" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2041" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2041" t="inlineStr"/>
-    </row>
-    <row r="2042">
-      <c r="A2042" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2042" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2042" t="inlineStr"/>
-    </row>
-    <row r="2043">
-      <c r="A2043" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2043" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2043" t="inlineStr"/>
-    </row>
-    <row r="2044">
-      <c r="A2044" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2044" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2044" t="inlineStr"/>
-    </row>
-    <row r="2045">
-      <c r="A2045" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2045" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2045" t="inlineStr"/>
-    </row>
-    <row r="2046">
-      <c r="A2046" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2046" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2046" t="inlineStr"/>
-    </row>
-    <row r="2047">
-      <c r="A2047" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2047" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2047" t="inlineStr"/>
-    </row>
-    <row r="2048">
-      <c r="A2048" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2048" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2048" t="inlineStr"/>
-    </row>
-    <row r="2049">
-      <c r="A2049" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2049" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2049" t="inlineStr"/>
-    </row>
-    <row r="2050">
-      <c r="A2050" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2050" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2050" t="inlineStr"/>
-    </row>
-    <row r="2051">
-      <c r="A2051" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2051" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2051" t="inlineStr"/>
-    </row>
-    <row r="2052">
-      <c r="A2052" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2052" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2052" t="inlineStr"/>
-    </row>
-    <row r="2053">
-      <c r="A2053" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2053" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2053" t="inlineStr"/>
-    </row>
-    <row r="2054">
-      <c r="A2054" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2054" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2054" t="inlineStr"/>
-    </row>
-    <row r="2055">
-      <c r="A2055" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2055" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2055" t="inlineStr"/>
-    </row>
-    <row r="2056">
-      <c r="A2056" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2056" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2056" t="inlineStr"/>
-    </row>
-    <row r="2057">
-      <c r="A2057" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2057" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2057" t="inlineStr"/>
-    </row>
-    <row r="2058">
-      <c r="A2058" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2058" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2058" t="inlineStr"/>
-    </row>
-    <row r="2059">
-      <c r="A2059" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2059" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2059" t="inlineStr"/>
-    </row>
-    <row r="2060">
-      <c r="A2060" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2060" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2060" t="inlineStr"/>
-    </row>
-    <row r="2061">
-      <c r="A2061" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2061" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2061" t="inlineStr"/>
-    </row>
-    <row r="2062">
-      <c r="A2062" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2062" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2062" t="inlineStr"/>
-    </row>
-    <row r="2063">
-      <c r="A2063" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2063" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2063" t="inlineStr"/>
-    </row>
-    <row r="2064">
-      <c r="A2064" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2064" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2064" t="inlineStr"/>
-    </row>
-    <row r="2065">
-      <c r="A2065" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2065" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2065" t="inlineStr"/>
-    </row>
-    <row r="2066">
-      <c r="A2066" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2066" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2066" t="inlineStr"/>
-    </row>
-    <row r="2067">
-      <c r="A2067" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2067" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2067" t="inlineStr"/>
-    </row>
-    <row r="2068">
-      <c r="A2068" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2068" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2068" t="inlineStr"/>
-    </row>
-    <row r="2069">
-      <c r="A2069" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2069" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2069" t="inlineStr"/>
-    </row>
-    <row r="2070">
-      <c r="A2070" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2070" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2070" t="inlineStr"/>
-    </row>
-    <row r="2071">
-      <c r="A2071" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2071" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2071" t="inlineStr"/>
-    </row>
-    <row r="2072">
-      <c r="A2072" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2072" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2072" t="inlineStr"/>
-    </row>
-    <row r="2073">
-      <c r="A2073" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2073" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2073" t="inlineStr"/>
-    </row>
-    <row r="2074">
-      <c r="A2074" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2074" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2074" t="inlineStr"/>
-    </row>
-    <row r="2075">
-      <c r="A2075" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2075" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2075" t="inlineStr"/>
-    </row>
-    <row r="2076">
-      <c r="A2076" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2076" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2076" t="inlineStr"/>
-    </row>
-    <row r="2077">
-      <c r="A2077" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2077" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2077" t="inlineStr"/>
-    </row>
-    <row r="2078">
-      <c r="A2078" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2078" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2078" t="inlineStr"/>
-    </row>
-    <row r="2079">
-      <c r="A2079" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2079" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2079" t="inlineStr"/>
-    </row>
-    <row r="2080">
-      <c r="A2080" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2080" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2080" t="inlineStr"/>
-    </row>
-    <row r="2081">
-      <c r="A2081" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2081" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2081" t="inlineStr"/>
-    </row>
-    <row r="2082">
-      <c r="A2082" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2082" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2082" t="inlineStr"/>
-    </row>
-    <row r="2083">
-      <c r="A2083" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2083" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2083" t="inlineStr"/>
-    </row>
-    <row r="2084">
-      <c r="A2084" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2084" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2084" t="inlineStr"/>
-    </row>
-    <row r="2085">
-      <c r="A2085" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2085" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2085" t="inlineStr"/>
-    </row>
-    <row r="2086">
-      <c r="A2086" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2086" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2086" t="inlineStr"/>
-    </row>
-    <row r="2087">
-      <c r="A2087" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2087" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2087" t="inlineStr"/>
-    </row>
-    <row r="2088">
-      <c r="A2088" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2088" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2088" t="inlineStr"/>
-    </row>
-    <row r="2089">
-      <c r="A2089" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2089" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2089" t="inlineStr"/>
-    </row>
-    <row r="2090">
-      <c r="A2090" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2090" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2090" t="inlineStr"/>
-    </row>
-    <row r="2091">
-      <c r="A2091" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2091" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2091" t="inlineStr"/>
-    </row>
-    <row r="2092">
-      <c r="A2092" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2092" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2092" t="inlineStr"/>
-    </row>
-    <row r="2093">
-      <c r="A2093" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2093" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2093" t="inlineStr"/>
-    </row>
-    <row r="2094">
-      <c r="A2094" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2094" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2094" t="inlineStr"/>
-    </row>
-    <row r="2095">
-      <c r="A2095" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2095" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2095" t="inlineStr"/>
-    </row>
-    <row r="2096">
-      <c r="A2096" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2096" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2096" t="inlineStr"/>
-    </row>
-    <row r="2097">
-      <c r="A2097" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2097" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2097" t="inlineStr"/>
-    </row>
-    <row r="2098">
-      <c r="A2098" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2098" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2098" t="inlineStr"/>
-    </row>
-    <row r="2099">
-      <c r="A2099" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2099" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2099" t="inlineStr"/>
-    </row>
-    <row r="2100">
-      <c r="A2100" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2100" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2100" t="inlineStr"/>
-    </row>
-    <row r="2101">
-      <c r="A2101" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2101" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2101" t="inlineStr"/>
-    </row>
-    <row r="2102">
-      <c r="A2102" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2102" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2102" t="inlineStr"/>
-    </row>
-    <row r="2103">
-      <c r="A2103" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2103" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2103" t="inlineStr"/>
-    </row>
-    <row r="2104">
-      <c r="A2104" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2104" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2104" t="inlineStr"/>
-    </row>
-    <row r="2105">
-      <c r="A2105" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2105" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2105" t="inlineStr"/>
-    </row>
-    <row r="2106">
-      <c r="A2106" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2106" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2106" t="inlineStr"/>
-    </row>
-    <row r="2107">
-      <c r="A2107" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2107" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2107" t="inlineStr"/>
-    </row>
-    <row r="2108">
-      <c r="A2108" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2108" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2108" t="inlineStr"/>
-    </row>
-    <row r="2109">
-      <c r="A2109" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2109" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2109" t="inlineStr"/>
-    </row>
-    <row r="2110">
-      <c r="A2110" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2110" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2110" t="inlineStr"/>
-    </row>
-    <row r="2111">
-      <c r="A2111" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2111" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2111" t="inlineStr"/>
-    </row>
-    <row r="2112">
-      <c r="A2112" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2112" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2112" t="inlineStr"/>
-    </row>
-    <row r="2113">
-      <c r="A2113" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2113" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2113" t="inlineStr"/>
-    </row>
-    <row r="2114">
-      <c r="A2114" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2114" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2114" t="inlineStr"/>
-    </row>
-    <row r="2115">
-      <c r="A2115" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2115" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2115" t="inlineStr"/>
-    </row>
-    <row r="2116">
-      <c r="A2116" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2116" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2116" t="inlineStr"/>
-    </row>
-    <row r="2117">
-      <c r="A2117" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2117" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2117" t="inlineStr"/>
-    </row>
-    <row r="2118">
-      <c r="A2118" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2118" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2118" t="inlineStr"/>
-    </row>
-    <row r="2119">
-      <c r="A2119" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2119" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2119" t="inlineStr"/>
-    </row>
-    <row r="2120">
-      <c r="A2120" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2120" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2120" t="inlineStr"/>
-    </row>
-    <row r="2121">
-      <c r="A2121" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2121" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2121" t="inlineStr"/>
-    </row>
-    <row r="2122">
-      <c r="A2122" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2122" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2122" t="inlineStr"/>
-    </row>
-    <row r="2123">
-      <c r="A2123" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2123" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2123" t="inlineStr"/>
-    </row>
-    <row r="2124">
-      <c r="A2124" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2124" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2124" t="inlineStr"/>
-    </row>
-    <row r="2125">
-      <c r="A2125" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2125" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2125" t="inlineStr"/>
-    </row>
-    <row r="2126">
-      <c r="A2126" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2126" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2126" t="inlineStr"/>
-    </row>
-    <row r="2127">
-      <c r="A2127" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2127" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2127" t="inlineStr"/>
-    </row>
-    <row r="2128">
-      <c r="A2128" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2128" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2128" t="inlineStr"/>
-    </row>
-    <row r="2129">
-      <c r="A2129" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2129" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2129" t="inlineStr"/>
-    </row>
-    <row r="2130">
-      <c r="A2130" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2130" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2130" t="inlineStr"/>
-    </row>
-    <row r="2131">
-      <c r="A2131" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2131" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2131" t="inlineStr"/>
-    </row>
-    <row r="2132">
-      <c r="A2132" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2132" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2132" t="inlineStr"/>
-    </row>
-    <row r="2133">
-      <c r="A2133" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2133" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2133" t="inlineStr"/>
-    </row>
-    <row r="2134">
-      <c r="A2134" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2134" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2134" t="inlineStr"/>
-    </row>
-    <row r="2135">
-      <c r="A2135" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2135" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2135" t="inlineStr"/>
-    </row>
-    <row r="2136">
-      <c r="A2136" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2136" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2136" t="inlineStr"/>
-    </row>
-    <row r="2137">
-      <c r="A2137" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2137" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2137" t="inlineStr"/>
-    </row>
-    <row r="2138">
-      <c r="A2138" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2138" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2138" t="inlineStr"/>
-    </row>
-    <row r="2139">
-      <c r="A2139" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2139" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2139" t="inlineStr"/>
-    </row>
-    <row r="2140">
-      <c r="A2140" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2140" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2140" t="inlineStr"/>
-    </row>
-    <row r="2141">
-      <c r="A2141" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2141" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2141" t="inlineStr"/>
-    </row>
-    <row r="2142">
-      <c r="A2142" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2142" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2142" t="inlineStr"/>
-    </row>
-    <row r="2143">
-      <c r="A2143" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2143" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2143" t="inlineStr"/>
-    </row>
-    <row r="2144">
-      <c r="A2144" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2144" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2144" t="inlineStr"/>
-    </row>
-    <row r="2145">
-      <c r="A2145" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2145" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2145" t="inlineStr"/>
-    </row>
-    <row r="2146">
-      <c r="A2146" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2146" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2146" t="inlineStr"/>
-    </row>
-    <row r="2147">
-      <c r="A2147" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2147" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2147" t="inlineStr"/>
-    </row>
-    <row r="2148">
-      <c r="A2148" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2148" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2148" t="inlineStr"/>
-    </row>
-    <row r="2149">
-      <c r="A2149" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2149" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2149" t="inlineStr"/>
-    </row>
-    <row r="2150">
-      <c r="A2150" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2150" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2150" t="inlineStr"/>
-    </row>
-    <row r="2151">
-      <c r="A2151" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2151" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2151" t="inlineStr"/>
-    </row>
-    <row r="2152">
-      <c r="A2152" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2152" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2152" t="inlineStr"/>
-    </row>
-    <row r="2153">
-      <c r="A2153" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2153" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2153" t="inlineStr"/>
-    </row>
-    <row r="2154">
-      <c r="A2154" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2154" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2154" t="inlineStr"/>
-    </row>
-    <row r="2155">
-      <c r="A2155" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2155" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2155" t="inlineStr"/>
-    </row>
-    <row r="2156">
-      <c r="A2156" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2156" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2156" t="inlineStr"/>
-    </row>
-    <row r="2157">
-      <c r="A2157" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2157" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2157" t="inlineStr"/>
-    </row>
-    <row r="2158">
-      <c r="A2158" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2158" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2158" t="inlineStr"/>
-    </row>
-    <row r="2159">
-      <c r="A2159" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2159" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2159" t="inlineStr"/>
-    </row>
-    <row r="2160">
-      <c r="A2160" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2160" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2160" t="inlineStr"/>
-    </row>
-    <row r="2161">
-      <c r="A2161" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2161" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2161" t="inlineStr"/>
-    </row>
-    <row r="2162">
-      <c r="A2162" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2162" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2162" t="inlineStr"/>
-    </row>
-    <row r="2163">
-      <c r="A2163" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2163" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2163" t="inlineStr"/>
-    </row>
-    <row r="2164">
-      <c r="A2164" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2164" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2164" t="inlineStr"/>
-    </row>
-    <row r="2165">
-      <c r="A2165" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2165" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2165" t="inlineStr"/>
-    </row>
-    <row r="2166">
-      <c r="A2166" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2166" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2166" t="inlineStr"/>
-    </row>
-    <row r="2167">
-      <c r="A2167" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2167" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2167" t="inlineStr"/>
-    </row>
-    <row r="2168">
-      <c r="A2168" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2168" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2168" t="inlineStr"/>
-    </row>
-    <row r="2169">
-      <c r="A2169" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2169" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2169" t="inlineStr"/>
-    </row>
-    <row r="2170">
-      <c r="A2170" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2170" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2170" t="inlineStr"/>
-    </row>
-    <row r="2171">
-      <c r="A2171" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2171" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2171" t="inlineStr"/>
-    </row>
-    <row r="2172">
-      <c r="A2172" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2172" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2172" t="inlineStr"/>
-    </row>
-    <row r="2173">
-      <c r="A2173" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2173" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2173" t="inlineStr"/>
-    </row>
-    <row r="2174">
-      <c r="A2174" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2174" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2174" t="inlineStr"/>
-    </row>
-    <row r="2175">
-      <c r="A2175" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2175" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2175" t="inlineStr"/>
-    </row>
-    <row r="2176">
-      <c r="A2176" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2176" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2176" t="inlineStr"/>
-    </row>
-    <row r="2177">
-      <c r="A2177" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2177" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2177" t="inlineStr"/>
-    </row>
-    <row r="2178">
-      <c r="A2178" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2178" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2178" t="inlineStr"/>
-    </row>
-    <row r="2179">
-      <c r="A2179" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2179" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2179" t="inlineStr"/>
-    </row>
-    <row r="2180">
-      <c r="A2180" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2180" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2180" t="inlineStr"/>
-    </row>
-    <row r="2181">
-      <c r="A2181" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2181" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2181" t="inlineStr"/>
-    </row>
-    <row r="2182">
-      <c r="A2182" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2182" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2182" t="inlineStr"/>
-    </row>
-    <row r="2183">
-      <c r="A2183" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2183" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2183" t="inlineStr"/>
-    </row>
-    <row r="2184">
-      <c r="A2184" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2184" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2184" t="inlineStr"/>
-    </row>
-    <row r="2185">
-      <c r="A2185" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2185" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2185" t="inlineStr"/>
-    </row>
-    <row r="2186">
-      <c r="A2186" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2186" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2186" t="inlineStr"/>
-    </row>
-    <row r="2187">
-      <c r="A2187" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2187" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2187" t="inlineStr"/>
-    </row>
-    <row r="2188">
-      <c r="A2188" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2188" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2188" t="inlineStr"/>
-    </row>
-    <row r="2189">
-      <c r="A2189" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2189" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2189" t="inlineStr"/>
-    </row>
-    <row r="2190">
-      <c r="A2190" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2190" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2190" t="inlineStr"/>
-    </row>
-    <row r="2191">
-      <c r="A2191" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2191" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2191" t="inlineStr"/>
-    </row>
-    <row r="2192">
-      <c r="A2192" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2192" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2192" t="inlineStr"/>
-    </row>
-    <row r="2193">
-      <c r="A2193" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2193" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2193" t="inlineStr"/>
-    </row>
-    <row r="2194">
-      <c r="A2194" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="B2194" t="inlineStr">
-        <is>
-          <t>nan nan</t>
-        </is>
-      </c>
-      <c r="C2194" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Route bad-phone rows to .review files with mapped output data
- Bad-phone rows go to campaign/customers .review files (same columns as main output)
- Fully empty rows dropped before processing (not routed to review)
- Duplicates dropped silently from main output only
</commit_message>
<xml_diff>
--- a/output/campaign_Otros_proyectos.xlsx
+++ b/output/campaign_Otros_proyectos.xlsx
@@ -4657,7 +4657,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jairo  Ramirez </t>
+          <t>Jairo  Ramirez</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
@@ -26332,7 +26332,7 @@
       </c>
       <c r="B1525" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jose Fernando Garcia Perez </t>
+          <t>Jose Fernando Garcia Perez</t>
         </is>
       </c>
       <c r="C1525" t="inlineStr">

</xml_diff>